<commit_message>
fix(sync): sinkronisasi rincian dinas cuti sakit izin antara dashboard dan ekspor excel resmi
</commit_message>
<xml_diff>
--- a/Rekapitulasi_Kehadiran_September_2026_Resmi.xlsx
+++ b/Rekapitulasi_Kehadiran_September_2026_Resmi.xlsx
@@ -2329,10 +2329,10 @@
       <c r="P15" s="75"/>
       <c r="Q15" s="83"/>
       <c r="R15" s="17"/>
-      <c r="S15" s="17"/>
-      <c r="T15" s="77">
+      <c r="S15" s="17">
         <v>2</v>
       </c>
+      <c r="T15" s="77"/>
       <c r="U15" s="83"/>
       <c r="V15" s="84"/>
       <c r="W15" s="19"/>
@@ -2690,10 +2690,10 @@
       <c r="P22" s="75"/>
       <c r="Q22" s="83"/>
       <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="77">
+      <c r="S22" s="17">
         <v>4</v>
       </c>
+      <c r="T22" s="77"/>
       <c r="U22" s="83"/>
       <c r="V22" s="84"/>
       <c r="W22" s="19"/>
@@ -2806,10 +2806,10 @@
       <c r="P24" s="75"/>
       <c r="Q24" s="83"/>
       <c r="R24" s="17"/>
-      <c r="S24" s="17"/>
-      <c r="T24" s="77">
+      <c r="S24" s="17">
         <v>5</v>
       </c>
+      <c r="T24" s="77"/>
       <c r="U24" s="83"/>
       <c r="V24" s="84"/>
       <c r="W24" s="19"/>
@@ -2862,10 +2862,10 @@
       <c r="P25" s="75"/>
       <c r="Q25" s="83"/>
       <c r="R25" s="17"/>
-      <c r="S25" s="17"/>
-      <c r="T25" s="77">
-        <v>1</v>
-      </c>
+      <c r="S25" s="17">
+        <v>1</v>
+      </c>
+      <c r="T25" s="77"/>
       <c r="U25" s="83"/>
       <c r="V25" s="84"/>
       <c r="W25" s="19"/>
@@ -2922,10 +2922,10 @@
       </c>
       <c r="Q26" s="83"/>
       <c r="R26" s="17"/>
-      <c r="S26" s="17"/>
-      <c r="T26" s="77">
+      <c r="S26" s="17">
         <v>11</v>
       </c>
+      <c r="T26" s="77"/>
       <c r="U26" s="83"/>
       <c r="V26" s="84"/>
       <c r="W26" s="19"/>
@@ -2978,10 +2978,10 @@
       <c r="P27" s="75"/>
       <c r="Q27" s="83"/>
       <c r="R27" s="17"/>
-      <c r="S27" s="17"/>
-      <c r="T27" s="77">
+      <c r="S27" s="17">
         <v>8</v>
       </c>
+      <c r="T27" s="77"/>
       <c r="U27" s="83"/>
       <c r="V27" s="84"/>
       <c r="W27" s="19"/>
@@ -3034,10 +3034,10 @@
       <c r="P28" s="75"/>
       <c r="Q28" s="83"/>
       <c r="R28" s="17"/>
-      <c r="S28" s="17"/>
-      <c r="T28" s="77">
+      <c r="S28" s="17">
         <v>11</v>
       </c>
+      <c r="T28" s="77"/>
       <c r="U28" s="83"/>
       <c r="V28" s="84"/>
       <c r="W28" s="19"/>
@@ -3090,10 +3090,10 @@
       <c r="P29" s="75"/>
       <c r="Q29" s="83"/>
       <c r="R29" s="17"/>
-      <c r="S29" s="17"/>
-      <c r="T29" s="77">
+      <c r="S29" s="17">
         <v>4</v>
       </c>
+      <c r="T29" s="77"/>
       <c r="U29" s="83"/>
       <c r="V29" s="84"/>
       <c r="W29" s="19"/>
@@ -3148,10 +3148,10 @@
       <c r="P30" s="75"/>
       <c r="Q30" s="83"/>
       <c r="R30" s="17"/>
-      <c r="S30" s="17"/>
-      <c r="T30" s="77">
+      <c r="S30" s="17">
         <v>2</v>
       </c>
+      <c r="T30" s="77"/>
       <c r="U30" s="83"/>
       <c r="V30" s="84"/>
       <c r="W30" s="19"/>
@@ -3204,10 +3204,10 @@
       <c r="P31" s="75"/>
       <c r="Q31" s="83"/>
       <c r="R31" s="17"/>
-      <c r="S31" s="17"/>
-      <c r="T31" s="77">
-        <v>1</v>
-      </c>
+      <c r="S31" s="17">
+        <v>1</v>
+      </c>
+      <c r="T31" s="77"/>
       <c r="U31" s="83"/>
       <c r="V31" s="84"/>
       <c r="W31" s="19"/>
@@ -3262,10 +3262,10 @@
       <c r="P32" s="75"/>
       <c r="Q32" s="83"/>
       <c r="R32" s="17"/>
-      <c r="S32" s="17"/>
-      <c r="T32" s="77">
+      <c r="S32" s="17">
         <v>16</v>
       </c>
+      <c r="T32" s="77"/>
       <c r="U32" s="83"/>
       <c r="V32" s="84"/>
       <c r="W32" s="19"/>
@@ -3322,10 +3322,10 @@
       </c>
       <c r="Q33" s="83"/>
       <c r="R33" s="17"/>
-      <c r="S33" s="17"/>
-      <c r="T33" s="77">
+      <c r="S33" s="17">
         <v>6</v>
       </c>
+      <c r="T33" s="77"/>
       <c r="U33" s="83"/>
       <c r="V33" s="84"/>
       <c r="W33" s="19"/>
@@ -3380,10 +3380,10 @@
       <c r="P34" s="75"/>
       <c r="Q34" s="83"/>
       <c r="R34" s="17"/>
-      <c r="S34" s="17"/>
-      <c r="T34" s="77">
+      <c r="S34" s="17">
         <v>5</v>
       </c>
+      <c r="T34" s="77"/>
       <c r="U34" s="83"/>
       <c r="V34" s="84"/>
       <c r="W34" s="19"/>
@@ -3438,10 +3438,10 @@
       </c>
       <c r="Q35" s="83"/>
       <c r="R35" s="17"/>
-      <c r="S35" s="17"/>
-      <c r="T35" s="77">
-        <v>1</v>
-      </c>
+      <c r="S35" s="17">
+        <v>1</v>
+      </c>
+      <c r="T35" s="77"/>
       <c r="U35" s="83"/>
       <c r="V35" s="84"/>
       <c r="W35" s="19"/>
@@ -3496,10 +3496,10 @@
       <c r="P36" s="75"/>
       <c r="Q36" s="83"/>
       <c r="R36" s="17"/>
-      <c r="S36" s="17"/>
-      <c r="T36" s="77">
+      <c r="S36" s="17">
         <v>8</v>
       </c>
+      <c r="T36" s="77"/>
       <c r="U36" s="83"/>
       <c r="V36" s="84"/>
       <c r="W36" s="19"/>
@@ -3552,10 +3552,10 @@
       <c r="P37" s="75"/>
       <c r="Q37" s="83"/>
       <c r="R37" s="17"/>
-      <c r="S37" s="17"/>
-      <c r="T37" s="77">
+      <c r="S37" s="17">
         <v>8</v>
       </c>
+      <c r="T37" s="77"/>
       <c r="U37" s="83"/>
       <c r="V37" s="84"/>
       <c r="W37" s="19"/>
@@ -3747,10 +3747,10 @@
       <c r="P41" s="75"/>
       <c r="Q41" s="83"/>
       <c r="R41" s="17"/>
-      <c r="S41" s="17"/>
-      <c r="T41" s="77">
+      <c r="S41" s="17">
         <v>8</v>
       </c>
+      <c r="T41" s="77"/>
       <c r="U41" s="83"/>
       <c r="V41" s="84"/>
       <c r="W41" s="19"/>
@@ -3892,10 +3892,10 @@
       <c r="P44" s="75"/>
       <c r="Q44" s="83"/>
       <c r="R44" s="17"/>
-      <c r="S44" s="17"/>
-      <c r="T44" s="77">
+      <c r="S44" s="17">
         <v>4</v>
       </c>
+      <c r="T44" s="77"/>
       <c r="U44" s="83"/>
       <c r="V44" s="84"/>
       <c r="W44" s="19"/>
@@ -4176,10 +4176,10 @@
       <c r="R50" s="17">
         <v>1</v>
       </c>
-      <c r="S50" s="17"/>
-      <c r="T50" s="77">
+      <c r="S50" s="17">
         <v>10</v>
       </c>
+      <c r="T50" s="77"/>
       <c r="U50" s="83"/>
       <c r="V50" s="84"/>
       <c r="W50" s="19"/>
@@ -4290,10 +4290,10 @@
       <c r="P52" s="75"/>
       <c r="Q52" s="83"/>
       <c r="R52" s="17"/>
-      <c r="S52" s="17"/>
-      <c r="T52" s="77">
-        <v>1</v>
-      </c>
+      <c r="S52" s="17">
+        <v>1</v>
+      </c>
+      <c r="T52" s="77"/>
       <c r="U52" s="83"/>
       <c r="V52" s="84"/>
       <c r="W52" s="19"/>
@@ -4402,10 +4402,10 @@
       <c r="P54" s="75"/>
       <c r="Q54" s="83"/>
       <c r="R54" s="17"/>
-      <c r="S54" s="17"/>
-      <c r="T54" s="77">
+      <c r="S54" s="17">
         <v>10</v>
       </c>
+      <c r="T54" s="77"/>
       <c r="U54" s="83"/>
       <c r="V54" s="84"/>
       <c r="W54" s="19"/>
@@ -4513,10 +4513,10 @@
       <c r="P56" s="75"/>
       <c r="Q56" s="83"/>
       <c r="R56" s="17"/>
-      <c r="S56" s="17"/>
-      <c r="T56" s="77">
+      <c r="S56" s="17">
         <v>8</v>
       </c>
+      <c r="T56" s="77"/>
       <c r="U56" s="83"/>
       <c r="V56" s="84"/>
       <c r="W56" s="19"/>
@@ -4656,10 +4656,10 @@
       <c r="P59" s="75"/>
       <c r="Q59" s="83"/>
       <c r="R59" s="17"/>
-      <c r="S59" s="17"/>
-      <c r="T59" s="77">
-        <v>1</v>
-      </c>
+      <c r="S59" s="17">
+        <v>1</v>
+      </c>
+      <c r="T59" s="77"/>
       <c r="U59" s="83"/>
       <c r="V59" s="84"/>
       <c r="W59" s="19"/>
@@ -4712,10 +4712,10 @@
       <c r="P60" s="75"/>
       <c r="Q60" s="83"/>
       <c r="R60" s="17"/>
-      <c r="S60" s="17"/>
-      <c r="T60" s="77">
+      <c r="S60" s="17">
         <v>4</v>
       </c>
+      <c r="T60" s="77"/>
       <c r="U60" s="83"/>
       <c r="V60" s="84"/>
       <c r="W60" s="19"/>
@@ -4855,10 +4855,10 @@
       <c r="P63" s="75"/>
       <c r="Q63" s="83"/>
       <c r="R63" s="17"/>
-      <c r="S63" s="17"/>
-      <c r="T63" s="77">
+      <c r="S63" s="17">
         <v>15</v>
       </c>
+      <c r="T63" s="77"/>
       <c r="U63" s="83"/>
       <c r="V63" s="84"/>
       <c r="W63" s="19"/>
@@ -4911,10 +4911,10 @@
       <c r="P64" s="75"/>
       <c r="Q64" s="83"/>
       <c r="R64" s="17"/>
-      <c r="S64" s="17"/>
-      <c r="T64" s="77">
+      <c r="S64" s="17">
         <v>9</v>
       </c>
+      <c r="T64" s="77"/>
       <c r="U64" s="83"/>
       <c r="V64" s="84"/>
       <c r="W64" s="19"/>
@@ -4969,10 +4969,10 @@
       <c r="P65" s="75"/>
       <c r="Q65" s="83"/>
       <c r="R65" s="17"/>
-      <c r="S65" s="17"/>
-      <c r="T65" s="77">
-        <v>1</v>
-      </c>
+      <c r="S65" s="17">
+        <v>1</v>
+      </c>
+      <c r="T65" s="77"/>
       <c r="U65" s="83"/>
       <c r="V65" s="84"/>
       <c r="W65" s="19"/>
@@ -5025,10 +5025,10 @@
       <c r="P66" s="75"/>
       <c r="Q66" s="83"/>
       <c r="R66" s="17"/>
-      <c r="S66" s="17"/>
-      <c r="T66" s="77">
+      <c r="S66" s="17">
         <v>8</v>
       </c>
+      <c r="T66" s="77"/>
       <c r="U66" s="83"/>
       <c r="V66" s="84"/>
       <c r="W66" s="19"/>
@@ -5137,10 +5137,10 @@
       <c r="R68" s="17">
         <v>1</v>
       </c>
-      <c r="S68" s="17"/>
-      <c r="T68" s="77">
+      <c r="S68" s="17">
         <v>8</v>
       </c>
+      <c r="T68" s="77"/>
       <c r="U68" s="83"/>
       <c r="V68" s="84"/>
       <c r="W68" s="19"/>
@@ -5193,10 +5193,10 @@
       <c r="P69" s="75"/>
       <c r="Q69" s="83"/>
       <c r="R69" s="17"/>
-      <c r="S69" s="17"/>
-      <c r="T69" s="77">
+      <c r="S69" s="17">
         <v>2</v>
       </c>
+      <c r="T69" s="77"/>
       <c r="U69" s="83"/>
       <c r="V69" s="84"/>
       <c r="W69" s="19"/>
@@ -5334,10 +5334,10 @@
       <c r="P72" s="75"/>
       <c r="Q72" s="83"/>
       <c r="R72" s="17"/>
-      <c r="S72" s="17"/>
-      <c r="T72" s="77">
+      <c r="S72" s="17">
         <v>8</v>
       </c>
+      <c r="T72" s="77"/>
       <c r="U72" s="83"/>
       <c r="V72" s="84"/>
       <c r="W72" s="19"/>
@@ -5475,10 +5475,10 @@
       <c r="P75" s="75"/>
       <c r="Q75" s="83"/>
       <c r="R75" s="17"/>
-      <c r="S75" s="17"/>
-      <c r="T75" s="77">
+      <c r="S75" s="17">
         <v>4</v>
       </c>
+      <c r="T75" s="77"/>
       <c r="U75" s="83"/>
       <c r="V75" s="84"/>
       <c r="W75" s="19"/>
@@ -5537,10 +5537,10 @@
       <c r="P76" s="75"/>
       <c r="Q76" s="83"/>
       <c r="R76" s="17"/>
-      <c r="S76" s="17"/>
-      <c r="T76" s="77">
-        <v>1</v>
-      </c>
+      <c r="S76" s="17">
+        <v>1</v>
+      </c>
+      <c r="T76" s="77"/>
       <c r="U76" s="83"/>
       <c r="V76" s="84"/>
       <c r="W76" s="19"/>
@@ -5593,10 +5593,10 @@
       <c r="P77" s="75"/>
       <c r="Q77" s="83"/>
       <c r="R77" s="17"/>
-      <c r="S77" s="17"/>
-      <c r="T77" s="77">
+      <c r="S77" s="17">
         <v>2</v>
       </c>
+      <c r="T77" s="77"/>
       <c r="U77" s="83"/>
       <c r="V77" s="84"/>
       <c r="W77" s="19"/>
@@ -5736,10 +5736,10 @@
       <c r="R80" s="17">
         <v>1</v>
       </c>
-      <c r="S80" s="17"/>
-      <c r="T80" s="77">
-        <v>1</v>
-      </c>
+      <c r="S80" s="17">
+        <v>1</v>
+      </c>
+      <c r="T80" s="77"/>
       <c r="U80" s="83"/>
       <c r="V80" s="84"/>
       <c r="W80" s="19"/>
@@ -6028,10 +6028,10 @@
       <c r="P86" s="75"/>
       <c r="Q86" s="83"/>
       <c r="R86" s="17"/>
-      <c r="S86" s="17"/>
-      <c r="T86" s="77">
+      <c r="S86" s="17">
         <v>4</v>
       </c>
+      <c r="T86" s="77"/>
       <c r="U86" s="83"/>
       <c r="V86" s="84"/>
       <c r="W86" s="19"/>
@@ -6086,10 +6086,10 @@
       <c r="P87" s="75"/>
       <c r="Q87" s="83"/>
       <c r="R87" s="17"/>
-      <c r="S87" s="17"/>
-      <c r="T87" s="77">
+      <c r="S87" s="17">
         <v>2</v>
       </c>
+      <c r="T87" s="77"/>
       <c r="U87" s="83"/>
       <c r="V87" s="84"/>
       <c r="W87" s="19"/>
@@ -6142,10 +6142,10 @@
       <c r="P88" s="75"/>
       <c r="Q88" s="83"/>
       <c r="R88" s="17"/>
-      <c r="S88" s="17"/>
-      <c r="T88" s="77">
+      <c r="S88" s="17">
         <v>5</v>
       </c>
+      <c r="T88" s="77"/>
       <c r="U88" s="83"/>
       <c r="V88" s="84"/>
       <c r="W88" s="19"/>
@@ -6200,10 +6200,10 @@
       <c r="P89" s="75"/>
       <c r="Q89" s="83"/>
       <c r="R89" s="17"/>
-      <c r="S89" s="17"/>
-      <c r="T89" s="77">
+      <c r="S89" s="17">
         <v>13</v>
       </c>
+      <c r="T89" s="77"/>
       <c r="U89" s="83"/>
       <c r="V89" s="84"/>
       <c r="W89" s="19"/>
@@ -6536,10 +6536,10 @@
       <c r="P96" s="75"/>
       <c r="Q96" s="83"/>
       <c r="R96" s="17"/>
-      <c r="S96" s="17"/>
-      <c r="T96" s="77">
+      <c r="S96" s="17">
         <v>4</v>
       </c>
+      <c r="T96" s="77"/>
       <c r="U96" s="83"/>
       <c r="V96" s="84"/>
       <c r="W96" s="19"/>
@@ -6596,10 +6596,10 @@
       </c>
       <c r="Q97" s="83"/>
       <c r="R97" s="17"/>
-      <c r="S97" s="17"/>
-      <c r="T97" s="77">
+      <c r="S97" s="17">
         <v>3</v>
       </c>
+      <c r="T97" s="77"/>
       <c r="U97" s="83"/>
       <c r="V97" s="84"/>
       <c r="W97" s="19"/>
@@ -6654,10 +6654,10 @@
       <c r="P98" s="75"/>
       <c r="Q98" s="83"/>
       <c r="R98" s="17"/>
-      <c r="S98" s="17"/>
-      <c r="T98" s="77">
+      <c r="S98" s="17">
         <v>2</v>
       </c>
+      <c r="T98" s="77"/>
       <c r="U98" s="83"/>
       <c r="V98" s="84"/>
       <c r="W98" s="19"/>
@@ -6710,10 +6710,10 @@
       <c r="P99" s="75"/>
       <c r="Q99" s="83"/>
       <c r="R99" s="17"/>
-      <c r="S99" s="17"/>
-      <c r="T99" s="77">
-        <v>1</v>
-      </c>
+      <c r="S99" s="17">
+        <v>1</v>
+      </c>
+      <c r="T99" s="77"/>
       <c r="U99" s="83"/>
       <c r="V99" s="84"/>
       <c r="W99" s="19"/>
@@ -6766,10 +6766,10 @@
       <c r="P100" s="75"/>
       <c r="Q100" s="83"/>
       <c r="R100" s="17"/>
-      <c r="S100" s="17"/>
-      <c r="T100" s="77">
+      <c r="S100" s="17">
         <v>2</v>
       </c>
+      <c r="T100" s="77"/>
       <c r="U100" s="83"/>
       <c r="V100" s="84"/>
       <c r="W100" s="19"/>
@@ -6820,9 +6820,7 @@
         <v>0</v>
       </c>
       <c r="N101" s="76"/>
-      <c r="O101" s="19">
-        <v>1</v>
-      </c>
+      <c r="O101" s="19"/>
       <c r="P101" s="75"/>
       <c r="Q101" s="83"/>
       <c r="R101" s="17"/>
@@ -6882,10 +6880,10 @@
       <c r="P102" s="75"/>
       <c r="Q102" s="83"/>
       <c r="R102" s="17"/>
-      <c r="S102" s="17"/>
-      <c r="T102" s="77">
-        <v>1</v>
-      </c>
+      <c r="S102" s="17">
+        <v>1</v>
+      </c>
+      <c r="T102" s="77"/>
       <c r="U102" s="83"/>
       <c r="V102" s="84"/>
       <c r="W102" s="19"/>
@@ -6938,10 +6936,10 @@
       <c r="P103" s="75"/>
       <c r="Q103" s="83"/>
       <c r="R103" s="17"/>
-      <c r="S103" s="17"/>
-      <c r="T103" s="77">
+      <c r="S103" s="17">
         <v>4</v>
       </c>
+      <c r="T103" s="77"/>
       <c r="U103" s="83"/>
       <c r="V103" s="84"/>
       <c r="W103" s="19"/>
@@ -7081,10 +7079,10 @@
       <c r="P106" s="75"/>
       <c r="Q106" s="83"/>
       <c r="R106" s="17"/>
-      <c r="S106" s="17"/>
-      <c r="T106" s="77">
+      <c r="S106" s="17">
         <v>13</v>
       </c>
+      <c r="T106" s="77"/>
       <c r="U106" s="83"/>
       <c r="V106" s="84"/>
       <c r="W106" s="19"/>
@@ -7222,10 +7220,10 @@
       <c r="P109" s="75"/>
       <c r="Q109" s="83"/>
       <c r="R109" s="17"/>
-      <c r="S109" s="17"/>
-      <c r="T109" s="77">
-        <v>1</v>
-      </c>
+      <c r="S109" s="17">
+        <v>1</v>
+      </c>
+      <c r="T109" s="77"/>
       <c r="U109" s="83"/>
       <c r="V109" s="84"/>
       <c r="W109" s="19"/>
@@ -7338,10 +7336,10 @@
       <c r="P111" s="75"/>
       <c r="Q111" s="83"/>
       <c r="R111" s="17"/>
-      <c r="S111" s="17"/>
-      <c r="T111" s="77">
+      <c r="S111" s="17">
         <v>4</v>
       </c>
+      <c r="T111" s="77"/>
       <c r="U111" s="83"/>
       <c r="V111" s="84"/>
       <c r="W111" s="19"/>
@@ -7396,10 +7394,10 @@
       <c r="P112" s="75"/>
       <c r="Q112" s="83"/>
       <c r="R112" s="17"/>
-      <c r="S112" s="17"/>
-      <c r="T112" s="77">
+      <c r="S112" s="17">
         <v>7</v>
       </c>
+      <c r="T112" s="77"/>
       <c r="U112" s="83"/>
       <c r="V112" s="84"/>
       <c r="W112" s="19"/>
@@ -7510,10 +7508,10 @@
       <c r="P114" s="75"/>
       <c r="Q114" s="83"/>
       <c r="R114" s="17"/>
-      <c r="S114" s="17"/>
-      <c r="T114" s="77">
+      <c r="S114" s="17">
         <v>3</v>
       </c>
+      <c r="T114" s="77"/>
       <c r="U114" s="83"/>
       <c r="V114" s="84"/>
       <c r="W114" s="19"/>
@@ -7566,10 +7564,10 @@
       <c r="P115" s="75"/>
       <c r="Q115" s="83"/>
       <c r="R115" s="17"/>
-      <c r="S115" s="17"/>
-      <c r="T115" s="77">
+      <c r="S115" s="17">
         <v>3</v>
       </c>
+      <c r="T115" s="77"/>
       <c r="U115" s="83"/>
       <c r="V115" s="84"/>
       <c r="W115" s="19"/>
@@ -7622,10 +7620,10 @@
       <c r="P116" s="75"/>
       <c r="Q116" s="83"/>
       <c r="R116" s="17"/>
-      <c r="S116" s="17"/>
-      <c r="T116" s="77">
+      <c r="S116" s="17">
         <v>15</v>
       </c>
+      <c r="T116" s="77"/>
       <c r="U116" s="83"/>
       <c r="V116" s="84"/>
       <c r="W116" s="19"/>
@@ -7680,10 +7678,10 @@
       <c r="P117" s="75"/>
       <c r="Q117" s="83"/>
       <c r="R117" s="17"/>
-      <c r="S117" s="17"/>
-      <c r="T117" s="77">
+      <c r="S117" s="17">
         <v>16</v>
       </c>
+      <c r="T117" s="77"/>
       <c r="U117" s="83"/>
       <c r="V117" s="84"/>
       <c r="W117" s="19"/>
@@ -7875,10 +7873,10 @@
       <c r="P121" s="75"/>
       <c r="Q121" s="83"/>
       <c r="R121" s="17"/>
-      <c r="S121" s="17"/>
-      <c r="T121" s="77">
-        <v>1</v>
-      </c>
+      <c r="S121" s="17">
+        <v>1</v>
+      </c>
+      <c r="T121" s="77"/>
       <c r="U121" s="83"/>
       <c r="V121" s="84"/>
       <c r="W121" s="19"/>
@@ -8041,10 +8039,10 @@
       <c r="P124" s="75"/>
       <c r="Q124" s="83"/>
       <c r="R124" s="17"/>
-      <c r="S124" s="17"/>
-      <c r="T124" s="77">
+      <c r="S124" s="17">
         <v>4</v>
       </c>
+      <c r="T124" s="77"/>
       <c r="U124" s="83"/>
       <c r="V124" s="84"/>
       <c r="W124" s="19"/>
@@ -8155,10 +8153,10 @@
       <c r="P126" s="75"/>
       <c r="Q126" s="83"/>
       <c r="R126" s="17"/>
-      <c r="S126" s="17"/>
-      <c r="T126" s="77">
-        <v>1</v>
-      </c>
+      <c r="S126" s="17">
+        <v>1</v>
+      </c>
+      <c r="T126" s="77"/>
       <c r="U126" s="83"/>
       <c r="V126" s="84"/>
       <c r="W126" s="19"/>
@@ -8211,10 +8209,10 @@
       <c r="P127" s="75"/>
       <c r="Q127" s="83"/>
       <c r="R127" s="17"/>
-      <c r="S127" s="17"/>
-      <c r="T127" s="77">
-        <v>1</v>
-      </c>
+      <c r="S127" s="17">
+        <v>1</v>
+      </c>
+      <c r="T127" s="77"/>
       <c r="U127" s="83"/>
       <c r="V127" s="84"/>
       <c r="W127" s="19"/>
@@ -8354,10 +8352,10 @@
       <c r="P130" s="75"/>
       <c r="Q130" s="83"/>
       <c r="R130" s="17"/>
-      <c r="S130" s="17"/>
-      <c r="T130" s="77">
+      <c r="S130" s="17">
         <v>5</v>
       </c>
+      <c r="T130" s="77"/>
       <c r="U130" s="83"/>
       <c r="V130" s="84"/>
       <c r="W130" s="19"/>
@@ -8464,10 +8462,10 @@
       <c r="P132" s="75"/>
       <c r="Q132" s="83"/>
       <c r="R132" s="17"/>
-      <c r="S132" s="17"/>
-      <c r="T132" s="77">
+      <c r="S132" s="17">
         <v>9</v>
       </c>
+      <c r="T132" s="77"/>
       <c r="U132" s="83"/>
       <c r="V132" s="84"/>
       <c r="W132" s="19"/>
@@ -8520,10 +8518,10 @@
       <c r="P133" s="75"/>
       <c r="Q133" s="83"/>
       <c r="R133" s="17"/>
-      <c r="S133" s="17"/>
-      <c r="T133" s="77">
+      <c r="S133" s="17">
         <v>11</v>
       </c>
+      <c r="T133" s="77"/>
       <c r="U133" s="83"/>
       <c r="V133" s="84"/>
       <c r="W133" s="19"/>
@@ -8688,10 +8686,10 @@
       <c r="P136" s="75"/>
       <c r="Q136" s="83"/>
       <c r="R136" s="17"/>
-      <c r="S136" s="17"/>
-      <c r="T136" s="77">
-        <v>1</v>
-      </c>
+      <c r="S136" s="17">
+        <v>1</v>
+      </c>
+      <c r="T136" s="77"/>
       <c r="U136" s="83"/>
       <c r="V136" s="84"/>
       <c r="W136" s="19"/>
@@ -8752,10 +8750,10 @@
       <c r="R137" s="17">
         <v>1</v>
       </c>
-      <c r="S137" s="17"/>
-      <c r="T137" s="77">
+      <c r="S137" s="17">
         <v>3</v>
       </c>
+      <c r="T137" s="77"/>
       <c r="U137" s="83"/>
       <c r="V137" s="84"/>
       <c r="W137" s="19"/>
@@ -9032,10 +9030,10 @@
       <c r="P142" s="75"/>
       <c r="Q142" s="83"/>
       <c r="R142" s="17"/>
-      <c r="S142" s="17"/>
-      <c r="T142" s="77">
+      <c r="S142" s="17">
         <v>9</v>
       </c>
+      <c r="T142" s="77"/>
       <c r="U142" s="83"/>
       <c r="V142" s="84"/>
       <c r="W142" s="19"/>
@@ -9146,10 +9144,10 @@
       <c r="P144" s="75"/>
       <c r="Q144" s="83"/>
       <c r="R144" s="17"/>
-      <c r="S144" s="17"/>
-      <c r="T144" s="77">
+      <c r="S144" s="17">
         <v>7</v>
       </c>
+      <c r="T144" s="77"/>
       <c r="U144" s="83"/>
       <c r="V144" s="84"/>
       <c r="W144" s="19"/>
@@ -9287,10 +9285,10 @@
       <c r="P147" s="75"/>
       <c r="Q147" s="83"/>
       <c r="R147" s="17"/>
-      <c r="S147" s="17"/>
-      <c r="T147" s="77">
+      <c r="S147" s="17">
         <v>16</v>
       </c>
+      <c r="T147" s="77"/>
       <c r="U147" s="83"/>
       <c r="V147" s="84"/>
       <c r="W147" s="19"/>
@@ -9451,10 +9449,10 @@
       <c r="P150" s="75"/>
       <c r="Q150" s="83"/>
       <c r="R150" s="17"/>
-      <c r="S150" s="17"/>
-      <c r="T150" s="77">
+      <c r="S150" s="17">
         <v>3</v>
       </c>
+      <c r="T150" s="77"/>
       <c r="U150" s="83"/>
       <c r="V150" s="84"/>
       <c r="W150" s="19"/>
@@ -9561,10 +9559,10 @@
       <c r="P152" s="75"/>
       <c r="Q152" s="83"/>
       <c r="R152" s="17"/>
-      <c r="S152" s="17"/>
-      <c r="T152" s="77">
-        <v>1</v>
-      </c>
+      <c r="S152" s="17">
+        <v>1</v>
+      </c>
+      <c r="T152" s="77"/>
       <c r="U152" s="83"/>
       <c r="V152" s="84"/>
       <c r="W152" s="19"/>
@@ -9619,10 +9617,10 @@
       <c r="P153" s="75"/>
       <c r="Q153" s="83"/>
       <c r="R153" s="17"/>
-      <c r="S153" s="17"/>
-      <c r="T153" s="77">
-        <v>1</v>
-      </c>
+      <c r="S153" s="17">
+        <v>1</v>
+      </c>
+      <c r="T153" s="77"/>
       <c r="U153" s="83"/>
       <c r="V153" s="84"/>
       <c r="W153" s="19"/>
@@ -9675,10 +9673,10 @@
       <c r="P154" s="75"/>
       <c r="Q154" s="83"/>
       <c r="R154" s="17"/>
-      <c r="S154" s="17"/>
-      <c r="T154" s="77">
+      <c r="S154" s="17">
         <v>2</v>
       </c>
+      <c r="T154" s="77"/>
       <c r="U154" s="83"/>
       <c r="V154" s="84"/>
       <c r="W154" s="19"/>
@@ -9731,10 +9729,10 @@
       <c r="P155" s="75"/>
       <c r="Q155" s="83"/>
       <c r="R155" s="17"/>
-      <c r="S155" s="17"/>
-      <c r="T155" s="77">
+      <c r="S155" s="17">
         <v>8</v>
       </c>
+      <c r="T155" s="77"/>
       <c r="U155" s="83"/>
       <c r="V155" s="84"/>
       <c r="W155" s="19"/>
@@ -10069,10 +10067,10 @@
       <c r="P162" s="75"/>
       <c r="Q162" s="83"/>
       <c r="R162" s="17"/>
-      <c r="S162" s="17"/>
-      <c r="T162" s="77">
+      <c r="S162" s="17">
         <v>4</v>
       </c>
+      <c r="T162" s="77"/>
       <c r="U162" s="83"/>
       <c r="V162" s="84"/>
       <c r="W162" s="19"/>
@@ -10372,10 +10370,10 @@
       <c r="P168" s="75"/>
       <c r="Q168" s="83"/>
       <c r="R168" s="17"/>
-      <c r="S168" s="17"/>
-      <c r="T168" s="77">
-        <v>1</v>
-      </c>
+      <c r="S168" s="17">
+        <v>1</v>
+      </c>
+      <c r="T168" s="77"/>
       <c r="U168" s="83"/>
       <c r="V168" s="84"/>
       <c r="W168" s="19"/>
@@ -10428,10 +10426,10 @@
       <c r="P169" s="75"/>
       <c r="Q169" s="83"/>
       <c r="R169" s="17"/>
-      <c r="S169" s="17"/>
-      <c r="T169" s="77">
-        <v>1</v>
-      </c>
+      <c r="S169" s="17">
+        <v>1</v>
+      </c>
+      <c r="T169" s="77"/>
       <c r="U169" s="83"/>
       <c r="V169" s="84"/>
       <c r="W169" s="19"/>

</xml_diff>